<commit_message>
fix(reconciliation): remove top duplicate alert and calibrate all sector demo datasets for 100% reconciliation
</commit_message>
<xml_diff>
--- a/demo_data/sectors/hizmet_yazilim/ap_aging.xlsx
+++ b/demo_data/sectors/hizmet_yazilim/ap_aging.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46042</v>
+        <v>46052</v>
       </c>
       <c r="D2" t="n">
-        <v>41661.37</v>
+        <v>40645.24</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -494,10 +494,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46052</v>
+        <v>46051</v>
       </c>
       <c r="D3" t="n">
-        <v>41661.37</v>
+        <v>40645.24</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46059</v>
+        <v>46063</v>
       </c>
       <c r="D4" t="n">
-        <v>69435.62</v>
+        <v>67742.06</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
         <v>46011</v>
       </c>
       <c r="D5" t="n">
-        <v>27774.25</v>
+        <v>54193.65</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tosyalı Çelik Profil Sanayi A.Ş.</t>
+          <t>Kordsa Teknik Tekstil A.Ş.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -563,10 +563,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46021</v>
+        <v>46067</v>
       </c>
       <c r="D6" t="n">
-        <v>27774.25</v>
+        <v>23709.72</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46075</v>
+        <v>46063</v>
       </c>
       <c r="D7" t="n">
-        <v>48604.93</v>
+        <v>23709.73</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -609,10 +609,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46036</v>
+        <v>46034</v>
       </c>
       <c r="D8" t="n">
-        <v>20830.68</v>
+        <v>40645.24</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aksa Akrilik Kimya Sanayii A.Ş.</t>
+          <t>Sasa Polyester Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46044</v>
+        <v>46067</v>
       </c>
       <c r="D9" t="n">
-        <v>20830.68</v>
+        <v>40645.24</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sasa Polyester Sanayi A.Ş.</t>
+          <t>Toros Tarım Sanayi ve Ticaret</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46075</v>
+        <v>46016</v>
       </c>
       <c r="D10" t="n">
-        <v>41661.37</v>
+        <v>16935.51</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46022</v>
+        <v>46019</v>
       </c>
       <c r="D11" t="n">
-        <v>34717.81</v>
+        <v>16935.52</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46056</v>
+        <v>46046</v>
       </c>
       <c r="D12" t="n">
-        <v>34717.81</v>
+        <v>33871.03</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46049</v>
+        <v>46053</v>
       </c>
       <c r="D13" t="n">
-        <v>17358.9</v>
+        <v>33871.03</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alkim Alkali Kimya A.Ş.</t>
+          <t>Tat Gıda Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46053</v>
+        <v>46013</v>
       </c>
       <c r="D14" t="n">
-        <v>17358.9</v>
+        <v>13548.42</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -770,10 +770,10 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46010</v>
+        <v>46003</v>
       </c>
       <c r="D15" t="n">
-        <v>27774.25</v>
+        <v>13548.41</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46028</v>
+        <v>46042</v>
       </c>
       <c r="D16" t="n">
-        <v>13887.12</v>
+        <v>13548.42</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>46029</v>
+        <v>46027</v>
       </c>
       <c r="D17" t="n">
-        <v>13887.12</v>
+        <v>13548.41</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46063</v>
+        <v>46070</v>
       </c>
       <c r="D18" t="n">
-        <v>27774.25</v>
+        <v>27096.83</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>46003</v>
+        <v>45997</v>
       </c>
       <c r="D19" t="n">
-        <v>12151.23</v>
+        <v>23709.72</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Borusan Mannesmann Boru A.Ş.</t>
+          <t>Sarkuysan Elektrolitik Bakır Sanayi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -885,10 +885,10 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46007</v>
+        <v>46086</v>
       </c>
       <c r="D20" t="n">
-        <v>12151.23</v>
+        <v>11854.86</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46077</v>
       </c>
       <c r="D21" t="n">
-        <v>12151.23</v>
+        <v>11854.86</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sarkuysan Elektrolitik Bakır Sanayi</t>
+          <t>Kastamonu Entegre Ağaç Sanayi</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -931,10 +931,10 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>46083</v>
+        <v>46037</v>
       </c>
       <c r="D22" t="n">
-        <v>12151.23</v>
+        <v>10161.31</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         <v>46035</v>
       </c>
       <c r="D23" t="n">
-        <v>20830.68</v>
+        <v>10161.31</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>46014</v>
+        <v>46011</v>
       </c>
       <c r="D24" t="n">
-        <v>10415.34</v>
+        <v>20322.62</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -991,7 +991,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Yıldız Entegre Ağaç Sanayi A.Ş.</t>
+          <t>Çamsan Ağaç Sanayi ve Ticaret</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1000,10 +1000,10 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>46013</v>
+        <v>46043</v>
       </c>
       <c r="D25" t="n">
-        <v>10415.34</v>
+        <v>16935.52</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1014,7 +1014,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Çamsan Ağaç Sanayi ve Ticaret</t>
+          <t>Ege Seramik Sanayi ve Ticaret</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1023,10 +1023,10 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>46044</v>
+        <v>46063</v>
       </c>
       <c r="D26" t="n">
-        <v>8679.450000000001</v>
+        <v>8467.76</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Çamsan Ağaç Sanayi ve Ticaret</t>
+          <t>Ege Seramik Sanayi ve Ticaret</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1046,10 +1046,10 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>46047</v>
+        <v>46060</v>
       </c>
       <c r="D27" t="n">
-        <v>8679.450000000001</v>
+        <v>8467.76</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ege Seramik Sanayi ve Ticaret</t>
+          <t>Kütahya Porselen Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1072,7 +1072,7 @@
         <v>46064</v>
       </c>
       <c r="D28" t="n">
-        <v>8679.450000000001</v>
+        <v>6774.2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1083,7 +1083,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ege Seramik Sanayi ve Ticaret</t>
+          <t>Kütahya Porselen Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1092,10 +1092,10 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>46066</v>
+        <v>46073</v>
       </c>
       <c r="D29" t="n">
-        <v>8679.450000000001</v>
+        <v>6774.21</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kütahya Porselen Sanayi A.Ş.</t>
+          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1115,10 +1115,10 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>46071</v>
+        <v>46026</v>
       </c>
       <c r="D30" t="n">
-        <v>6943.56</v>
+        <v>6774.2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Kütahya Porselen Sanayi A.Ş.</t>
+          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1138,10 +1138,10 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>46070</v>
+        <v>46019</v>
       </c>
       <c r="D31" t="n">
-        <v>6943.56</v>
+        <v>6774.21</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
+          <t>DYO Boya Fabrikaları Sanayi A.Ş.</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1161,10 +1161,10 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>46027</v>
+        <v>46036</v>
       </c>
       <c r="D32" t="n">
-        <v>6943.56</v>
+        <v>10161.31</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
+          <t>Polisan Holding Kimya Sanayi</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1184,10 +1184,10 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>46026</v>
+        <v>46043</v>
       </c>
       <c r="D33" t="n">
-        <v>6943.56</v>
+        <v>10161.31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DYO Boya Fabrikaları Sanayi A.Ş.</t>
+          <t>Filli Boya Betek Boya ve Kimya</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1207,104 +1207,12 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>46042</v>
+        <v>46059</v>
       </c>
       <c r="D34" t="n">
-        <v>10415.34</v>
+        <v>10161.3</v>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Polisan Holding Kimya Sanayi</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>BL-2034</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>46048</v>
-      </c>
-      <c r="D35" t="n">
-        <v>5207.67</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Polisan Holding Kimya Sanayi</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>BL-2035</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>46053</v>
-      </c>
-      <c r="D36" t="n">
-        <v>5207.67</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Filli Boya Betek Boya ve Kimya</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>BL-2036</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>46060</v>
-      </c>
-      <c r="D37" t="n">
-        <v>5207.67</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Filli Boya Betek Boya ve Kimya</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>BL-2037</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>46048</v>
-      </c>
-      <c r="D38" t="n">
-        <v>5207.67</v>
-      </c>
-      <c r="E38" t="inlineStr">
         <is>
           <t>TL</t>
         </is>

</xml_diff>

<commit_message>
feat(ux): streamline hero demo to prominent sector showcase, unify upload into single smart dropzone, and expand to 7 reconciled industry datasets
</commit_message>
<xml_diff>
--- a/demo_data/sectors/hizmet_yazilim/ap_aging.xlsx
+++ b/demo_data/sectors/hizmet_yazilim/ap_aging.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>İsdemir İskenderun Demir Çelik A.Ş.</t>
+          <t>Amazon Web Services (AWS) EMEA Sarl</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46052</v>
+        <v>46045</v>
       </c>
       <c r="D2" t="n">
-        <v>40645.24</v>
+        <v>194419.72</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -485,7 +485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>İsdemir İskenderun Demir Çelik A.Ş.</t>
+          <t>Microsoft İrlanda Bulut Lisanslama</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,10 +494,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46051</v>
+        <v>46049</v>
       </c>
       <c r="D3" t="n">
-        <v>40645.24</v>
+        <v>166645.48</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -508,7 +508,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Erdemir Ereğli Demir ve Çelik A.Ş.</t>
+          <t>Google Cloud Bilgi Teknolojileri</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46063</v>
+        <v>46009</v>
       </c>
       <c r="D4" t="n">
-        <v>67742.06</v>
+        <v>124984.11</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tosyalı Çelik Profil Sanayi A.Ş.</t>
+          <t>MongoDB Inc. Bulut Veritabanı Hizmeti</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46011</v>
+        <v>46048</v>
       </c>
       <c r="D5" t="n">
-        <v>54193.65</v>
+        <v>55548.49</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kordsa Teknik Tekstil A.Ş.</t>
+          <t>Cloudflare Inc. Güvenlik ve CDN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -563,10 +563,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46067</v>
+        <v>46063</v>
       </c>
       <c r="D6" t="n">
-        <v>23709.72</v>
+        <v>20830.69</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kordsa Teknik Tekstil A.Ş.</t>
+          <t>Cloudflare Inc. Güvenlik ve CDN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46063</v>
+        <v>46069</v>
       </c>
       <c r="D7" t="n">
-        <v>23709.73</v>
+        <v>20830.68</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aksa Akrilik Kimya Sanayii A.Ş.</t>
+          <t>Datadog Altyapı İzleme Sistemleri</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -609,10 +609,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46034</v>
+        <v>46049</v>
       </c>
       <c r="D8" t="n">
-        <v>40645.24</v>
+        <v>34717.81</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sasa Polyester Sanayi A.Ş.</t>
+          <t>Atlassian Jira / Confluence Kurumsal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46067</v>
+        <v>46019</v>
       </c>
       <c r="D9" t="n">
-        <v>40645.24</v>
+        <v>13887.12</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Toros Tarım Sanayi ve Ticaret</t>
+          <t>Atlassian Jira / Confluence Kurumsal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46016</v>
+        <v>46018</v>
       </c>
       <c r="D10" t="n">
-        <v>16935.51</v>
+        <v>13887.13</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Toros Tarım Sanayi ve Ticaret</t>
+          <t>Slack Technologies Kurumsal İletişim</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46019</v>
+        <v>46031</v>
       </c>
       <c r="D11" t="n">
-        <v>16935.52</v>
+        <v>20830.68</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gentaş Kimya Sanayi Pazarlama</t>
+          <t>JetBrains Geliştirici Ortamı Araçları</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46046</v>
+        <v>46059</v>
       </c>
       <c r="D12" t="n">
-        <v>33871.03</v>
+        <v>6943.56</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Alkim Alkali Kimya A.Ş.</t>
+          <t>JetBrains Geliştirici Ortamı Araçları</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46053</v>
+        <v>46062</v>
       </c>
       <c r="D13" t="n">
-        <v>33871.03</v>
+        <v>6943.56</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tat Gıda Sanayi A.Ş.</t>
+          <t>Twilio SMS &amp; İletişim Gateway</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46013</v>
+        <v>46064</v>
       </c>
       <c r="D14" t="n">
-        <v>13548.42</v>
+        <v>6943.56</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -761,7 +761,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tat Gıda Sanayi A.Ş.</t>
+          <t>Twilio SMS &amp; İletişim Gateway</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -770,449 +770,12 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46003</v>
+        <v>46066</v>
       </c>
       <c r="D15" t="n">
-        <v>13548.41</v>
+        <v>6943.57</v>
       </c>
       <c r="E15" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Pınar Süt Mamülleri Sanayii A.Ş.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BL-2015</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>46042</v>
-      </c>
-      <c r="D16" t="n">
-        <v>13548.42</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Pınar Süt Mamülleri Sanayii A.Ş.</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>BL-2016</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>46027</v>
-      </c>
-      <c r="D17" t="n">
-        <v>13548.41</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Banvit Bandırma Vitaminli Yem</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>BL-2017</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>46070</v>
-      </c>
-      <c r="D18" t="n">
-        <v>27096.83</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Borusan Mannesmann Boru A.Ş.</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>BL-2018</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>45997</v>
-      </c>
-      <c r="D19" t="n">
-        <v>23709.72</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Sarkuysan Elektrolitik Bakır Sanayi</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BL-2019</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>46086</v>
-      </c>
-      <c r="D20" t="n">
-        <v>11854.86</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Sarkuysan Elektrolitik Bakır Sanayi</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>BL-2020</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>46077</v>
-      </c>
-      <c r="D21" t="n">
-        <v>11854.86</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Kastamonu Entegre Ağaç Sanayi</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BL-2021</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D22" t="n">
-        <v>10161.31</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Kastamonu Entegre Ağaç Sanayi</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>BL-2022</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>46035</v>
-      </c>
-      <c r="D23" t="n">
-        <v>10161.31</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Yıldız Entegre Ağaç Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>BL-2023</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>46011</v>
-      </c>
-      <c r="D24" t="n">
-        <v>20322.62</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Çamsan Ağaç Sanayi ve Ticaret</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>BL-2024</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>46043</v>
-      </c>
-      <c r="D25" t="n">
-        <v>16935.52</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Ege Seramik Sanayi ve Ticaret</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>BL-2025</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>46063</v>
-      </c>
-      <c r="D26" t="n">
-        <v>8467.76</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Ege Seramik Sanayi ve Ticaret</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>BL-2026</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>46060</v>
-      </c>
-      <c r="D27" t="n">
-        <v>8467.76</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Kütahya Porselen Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>BL-2027</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>46064</v>
-      </c>
-      <c r="D28" t="n">
-        <v>6774.2</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Kütahya Porselen Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>BL-2028</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>46073</v>
-      </c>
-      <c r="D29" t="n">
-        <v>6774.21</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>BL-2029</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>46026</v>
-      </c>
-      <c r="D30" t="n">
-        <v>6774.2</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Akzo Nobel Boya Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>BL-2030</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>46019</v>
-      </c>
-      <c r="D31" t="n">
-        <v>6774.21</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>DYO Boya Fabrikaları Sanayi A.Ş.</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>BL-2031</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>46036</v>
-      </c>
-      <c r="D32" t="n">
-        <v>10161.31</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Polisan Holding Kimya Sanayi</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>BL-2032</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>46043</v>
-      </c>
-      <c r="D33" t="n">
-        <v>10161.31</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Filli Boya Betek Boya ve Kimya</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>BL-2033</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>46059</v>
-      </c>
-      <c r="D34" t="n">
-        <v>10161.3</v>
-      </c>
-      <c r="E34" t="inlineStr">
         <is>
           <t>TL</t>
         </is>

</xml_diff>